<commit_message>
try a judge prompt to test accuracy of reasoning of first prompt response
</commit_message>
<xml_diff>
--- a/output/df_small_negatives.xlsx
+++ b/output/df_small_negatives.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,6 +481,11 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>filter_reason</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>alt_abbrev_response</t>
         </is>
       </c>
@@ -488,32 +493,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HGNC:24086</t>
+          <t>HGNC:14758</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ENSG00000148584</t>
+          <t>ENSG00000176510, ENSG00000285252</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GENE ID:29974</t>
+          <t>GENE ID:392133</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>A1CF</t>
+          <t>OR10AC1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ACF64</t>
+          <t>OR10AC1P</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>APOBEC1 complementation factor</t>
+          <t>olfactory receptor family 10 subfamily AC member 1 (gene/pseudogene)</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -521,37 +526,22 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
-    Inputs:
-    Alias gene symbol: ACF64
-    HGNC record ID: HGNC:24086
-    Primary gene symbol: A1CF
-    Official HGNC gene name: APOBEC1 complementation factor
-    Task:
-    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
-    or a nearly identical wording, while still uniquely identifying the same gene. 
-    2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
-    3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
-    through the removal of select characters. 
-    Special case: 
-    Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not Alternate Abbreviations 
-    while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
-    Exclusion Criteria:
-    1. If an alias symbol contains numerical characters not present in the primary gene symbol 
-    or official gene name, it should NOT be classified as an Alternate Abbreviation no matter what criteria it meets.
-    2. Aliases derived from historical protein names, molecular weights (e.g., numbers representing 
-    protein size), biochemical characterizations, or gene family names should NOT be considered Alternate Abbreviations.
-    Examples:
-    1-
-    Alias gene symbol: ACF65
-    Official HGNC gene name: APOBEC1 complementation factor
-    Primary gene symbol: A1CF
-    2-
-    Alias gene symbol: ALPHA4GNT
-    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
-    Primary gene symbol: A4GNT
+          <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
+    You will get fired if your accuracy is less than 95%.
+    Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
+    the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
+    of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
+    have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
+    gene name provided in the prompt. Keep in mind, a gene name with a number after the name is not the same gene as a gene name 
+    with no numbers or different numbers after the name.
+    Task: Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. Give a one sentence reason for
+    your determination.
+    Here is the gene information:
+    Alias gene symbol: OR10AC1P
+    HGNC record ID: HGNC:14758
+    Primary gene symbol: OR10AC1
+    Official HGNC gene name: olfactory receptor family 10 subfamily AC member 1 (gene/pseudogene)
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -560,27 +550,27 @@
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id":"HGNC:24086"
-    "alias_symbol": "ACF64",
-    "primary_gene_symbol": "A1CF",
-    "name": "APOBEC1 complementation factor",
+    "reason": statement,
     "alternate_abbreviation": "TRUE or FALSE"
-    }</t>
+    }
+    </t>
         </is>
       </c>
       <c r="I2" t="b">
         <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6</v>
+        <v>0.875</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>passed_filters</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>{
-"hgnc_id": "HGNC:24086",
-"alias_symbol": "ACF64",
-"primary_gene_symbol": "A1CF",
-"name": "APOBEC1 complementation factor",
+"reason": "The alias symbol OR10AC1P is not an alternate abbreviation because it includes an additional 'P' at the end, which is not present in the official gene name or primary symbol and likely indicates a pseudogene designation.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -589,32 +579,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HGNC:318</t>
+          <t>HGNC:14875</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ENSG00000038002</t>
+          <t>ENSG00000132704</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GENE ID:175</t>
+          <t>GENE ID:79368</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AGA</t>
+          <t>FCRL2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ASRG</t>
+          <t>FCRH2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>aspartylglucosaminidase</t>
+          <t>Fc receptor like 2</t>
         </is>
       </c>
       <c r="G3" t="b">
@@ -622,37 +612,22 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
-    Inputs:
-    Alias gene symbol: ASRG
-    HGNC record ID: HGNC:318
-    Primary gene symbol: AGA
-    Official HGNC gene name: aspartylglucosaminidase
-    Task:
-    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
-    or a nearly identical wording, while still uniquely identifying the same gene. 
-    2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
-    3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
-    through the removal of select characters. 
-    Special case: 
-    Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not Alternate Abbreviations 
-    while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
-    Exclusion Criteria:
-    1. If an alias symbol contains numerical characters not present in the primary gene symbol 
-    or official gene name, it should NOT be classified as an Alternate Abbreviation no matter what criteria it meets.
-    2. Aliases derived from historical protein names, molecular weights (e.g., numbers representing 
-    protein size), biochemical characterizations, or gene family names should NOT be considered Alternate Abbreviations.
-    Examples:
-    1-
-    Alias gene symbol: ACF65
-    Official HGNC gene name: APOBEC1 complementation factor
-    Primary gene symbol: A1CF
-    2-
-    Alias gene symbol: ALPHA4GNT
-    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
-    Primary gene symbol: A4GNT
+          <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
+    You will get fired if your accuracy is less than 95%.
+    Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
+    the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
+    of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
+    have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
+    gene name provided in the prompt. Keep in mind, a gene name with a number after the name is not the same gene as a gene name 
+    with no numbers or different numbers after the name.
+    Task: Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. Give a one sentence reason for
+    your determination.
+    Here is the gene information:
+    Alias gene symbol: FCRH2
+    HGNC record ID: HGNC:14875
+    Primary gene symbol: FCRL2
+    Official HGNC gene name: Fc receptor like 2
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -661,27 +636,27 @@
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id":"HGNC:318"
-    "alias_symbol": "ASRG",
-    "primary_gene_symbol": "AGA",
-    "name": "aspartylglucosaminidase",
+    "reason": statement,
     "alternate_abbreviation": "TRUE or FALSE"
-    }</t>
+    }
+    </t>
         </is>
       </c>
       <c r="I3" t="b">
         <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>passed_filters</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>{
-"hgnc_id":"HGNC:318",
-"alias_symbol": "ASRG",
-"primary_gene_symbol": "AGA",
-"name": "aspartylglucosaminidase",
+"reason": "FCRH2 is not an alternate abbreviation of 'Fc receptor like 2' as it contains an 'H' which is not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -690,32 +665,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HGNC:3308</t>
+          <t>HGNC:20014</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ENSG00000139610</t>
+          <t>ENSG00000180189</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GENE ID:1990</t>
+          <t>GENE ID:319130</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CELA1</t>
+          <t>HMGB1P14</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ELA1</t>
+          <t>HMGB1L14</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>chymotrypsin like elastase 1</t>
+          <t>high mobility group box 1 pseudogene 14</t>
         </is>
       </c>
       <c r="G4" t="b">
@@ -723,37 +698,22 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
-    Inputs:
-    Alias gene symbol: ELA1
-    HGNC record ID: HGNC:3308
-    Primary gene symbol: CELA1
-    Official HGNC gene name: chymotrypsin like elastase 1
-    Task:
-    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
-    or a nearly identical wording, while still uniquely identifying the same gene. 
-    2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
-    3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
-    through the removal of select characters. 
-    Special case: 
-    Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not Alternate Abbreviations 
-    while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
-    Exclusion Criteria:
-    1. If an alias symbol contains numerical characters not present in the primary gene symbol 
-    or official gene name, it should NOT be classified as an Alternate Abbreviation no matter what criteria it meets.
-    2. Aliases derived from historical protein names, molecular weights (e.g., numbers representing 
-    protein size), biochemical characterizations, or gene family names should NOT be considered Alternate Abbreviations.
-    Examples:
-    1-
-    Alias gene symbol: ACF65
-    Official HGNC gene name: APOBEC1 complementation factor
-    Primary gene symbol: A1CF
-    2-
-    Alias gene symbol: ALPHA4GNT
-    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
-    Primary gene symbol: A4GNT
+          <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
+    You will get fired if your accuracy is less than 95%.
+    Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
+    the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
+    of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
+    have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
+    gene name provided in the prompt. Keep in mind, a gene name with a number after the name is not the same gene as a gene name 
+    with no numbers or different numbers after the name.
+    Task: Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. Give a one sentence reason for
+    your determination.
+    Here is the gene information:
+    Alias gene symbol: HMGB1L14
+    HGNC record ID: HGNC:20014
+    Primary gene symbol: HMGB1P14
+    Official HGNC gene name: high mobility group box 1 pseudogene 14
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -762,27 +722,27 @@
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id":"HGNC:3308"
-    "alias_symbol": "ELA1",
-    "primary_gene_symbol": "CELA1",
-    "name": "chymotrypsin like elastase 1",
+    "reason": statement,
     "alternate_abbreviation": "TRUE or FALSE"
-    }</t>
+    }
+    </t>
         </is>
       </c>
       <c r="I4" t="b">
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8</v>
+        <v>0.875</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>passed_filters</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>{
-"hgnc_id":"HGNC:3308",
-"alias_symbol": "ELA1",
-"primary_gene_symbol": "CELA1",
-"name": "chymotrypsin like elastase 1",
+"reason": "The alias symbol HMGB1L14 is not an alternate abbreviation because it uses 'L' instead of 'P' to represent 'pseudogene', which is a different character not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -791,32 +751,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HGNC:42171</t>
+          <t>HGNC:318</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ENSG00000232928</t>
+          <t>ENSG00000038002</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GENE ID:100133180</t>
+          <t>GENE ID:175</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DDX3P1</t>
+          <t>AGA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DDX3YP1</t>
+          <t>ASRG</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>DEAD-box helicase 3 pseudogene 1</t>
+          <t>aspartylglucosaminidase</t>
         </is>
       </c>
       <c r="G5" t="b">
@@ -824,37 +784,22 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
-    Inputs:
-    Alias gene symbol: DDX3YP1
-    HGNC record ID: HGNC:42171
-    Primary gene symbol: DDX3P1
-    Official HGNC gene name: DEAD-box helicase 3 pseudogene 1
-    Task:
-    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
-    or a nearly identical wording, while still uniquely identifying the same gene. 
-    2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
-    3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
-    through the removal of select characters. 
-    Special case: 
-    Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not Alternate Abbreviations 
-    while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
-    Exclusion Criteria:
-    1. If an alias symbol contains numerical characters not present in the primary gene symbol 
-    or official gene name, it should NOT be classified as an Alternate Abbreviation no matter what criteria it meets.
-    2. Aliases derived from historical protein names, molecular weights (e.g., numbers representing 
-    protein size), biochemical characterizations, or gene family names should NOT be considered Alternate Abbreviations.
-    Examples:
-    1-
-    Alias gene symbol: ACF65
-    Official HGNC gene name: APOBEC1 complementation factor
-    Primary gene symbol: A1CF
-    2-
-    Alias gene symbol: ALPHA4GNT
-    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
-    Primary gene symbol: A4GNT
+          <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
+    You will get fired if your accuracy is less than 95%.
+    Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
+    the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
+    of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
+    have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
+    gene name provided in the prompt. Keep in mind, a gene name with a number after the name is not the same gene as a gene name 
+    with no numbers or different numbers after the name.
+    Task: Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. Give a one sentence reason for
+    your determination.
+    Here is the gene information:
+    Alias gene symbol: ASRG
+    HGNC record ID: HGNC:318
+    Primary gene symbol: AGA
+    Official HGNC gene name: aspartylglucosaminidase
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
@@ -863,27 +808,27 @@
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id":"HGNC:42171"
-    "alias_symbol": "DDX3YP1",
-    "primary_gene_symbol": "DDX3P1",
-    "name": "DEAD-box helicase 3 pseudogene 1",
+    "reason": statement,
     "alternate_abbreviation": "TRUE or FALSE"
-    }</t>
+    }
+    </t>
         </is>
       </c>
       <c r="I5" t="b">
         <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8571428571428572</v>
+        <v>0.5</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>passed_filters</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>{
-"hgnc_id":"HGNC:42171",
-"alias_symbol": "DDX3YP1",
-"primary_gene_symbol": "DDX3P1",
-"name": "DEAD-box helicase 3 pseudogene 1",
+"reason": "ASRG is not an alternate abbreviation of aspartylglucosaminidase as it contains an 'S' which is not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>

</xml_diff>